<commit_message>
feat: board seats, rebuilt import, shared tables and app header
</commit_message>
<xml_diff>
--- a/apps/server/samples/marlowe-stakeholder-report.xlsx
+++ b/apps/server/samples/marlowe-stakeholder-report.xlsx
@@ -794,22 +794,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Larkspur Ventures Fund II, L.P.</t>
+          <t xml:space="preserve">Corinne Ashdown</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ir@larkspur.example</t>
+          <t xml:space="preserve">corinne@larkspur.example</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fund</t>
+          <t xml:space="preserve">Individual</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Investor</t>
+          <t xml:space="preserve">Board member</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partner, Larkspur Ventures</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-05-03</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -819,19 +829,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE</t>
+          <t xml:space="preserve">CA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tidewater Seed Partners</t>
+          <t xml:space="preserve">Larkspur Ventures Fund II, L.P.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">deals@tidewater.example</t>
+          <t xml:space="preserve">ir@larkspur.example</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -858,17 +868,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alder Grove Capital SPV</t>
+          <t xml:space="preserve">Tidewater Seed Partners</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">spv@aldergrove.example</t>
+          <t xml:space="preserve">deals@tidewater.example</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entity</t>
+          <t xml:space="preserve">Fund</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -890,12 +900,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beacon Street Angels LLC</t>
+          <t xml:space="preserve">Alder Grove Capital SPV</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">hello@beaconstreet.example</t>
+          <t xml:space="preserve">spv@aldergrove.example</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -915,19 +925,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">MA</t>
+          <t xml:space="preserve">DE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Summit Ridge Family Office</t>
+          <t xml:space="preserve">Beacon Street Angels LLC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">office@summitridge.example</t>
+          <t xml:space="preserve">hello@beaconstreet.example</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -947,24 +957,24 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">CO</t>
+          <t xml:space="preserve">MA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Orbital Founders Fund</t>
+          <t xml:space="preserve">Summit Ridge Family Office</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">team@orbitalff.example</t>
+          <t xml:space="preserve">office@summitridge.example</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fund</t>
+          <t xml:space="preserve">Entity</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -979,19 +989,19 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">CA</t>
+          <t xml:space="preserve">CO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobalt Bay Ventures</t>
+          <t xml:space="preserve">Orbital Founders Fund</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ir@cobaltbay.example</t>
+          <t xml:space="preserve">team@orbitalff.example</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1018,17 +1028,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quill &amp; Compass Holdings</t>
+          <t xml:space="preserve">Cobalt Bay Ventures</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">invest@quillcompass.example</t>
+          <t xml:space="preserve">ir@cobaltbay.example</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entity</t>
+          <t xml:space="preserve">Fund</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1043,24 +1053,24 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">NY</t>
+          <t xml:space="preserve">CA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wren Capital</t>
+          <t xml:space="preserve">Quill &amp; Compass Holdings</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">partners@wren.example</t>
+          <t xml:space="preserve">invest@quillcompass.example</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fund</t>
+          <t xml:space="preserve">Entity</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1075,24 +1085,24 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve">DE</t>
+          <t xml:space="preserve">NY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dev Anand</t>
+          <t xml:space="preserve">Wren Capital</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">dev.anand@mail.example</t>
+          <t xml:space="preserve">partners@wren.example</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Individual</t>
+          <t xml:space="preserve">Fund</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1100,11 +1110,6 @@
           <t xml:space="preserve">Investor</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Angel investor</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t xml:space="preserve">US</t>
@@ -1112,19 +1117,19 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">CA</t>
+          <t xml:space="preserve">DE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Priyanka Nair</t>
+          <t xml:space="preserve">Dev Anand</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">priyanka.nair@mail.example</t>
+          <t xml:space="preserve">dev.anand@mail.example</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1149,37 +1154,74 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WA</t>
+          <t xml:space="preserve">CA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">Priyanka Nair</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">priyanka.nair@mail.example</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individual</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investor</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Angel investor</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t xml:space="preserve">Samuel Oduya</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Individual</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individual</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">Investor</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t xml:space="preserve">Angel investor</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">US</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t xml:space="preserve">GA</t>
         </is>

</xml_diff>